<commit_message>
Update status batch one done
</commit_message>
<xml_diff>
--- a/Projects_Section_Wise.xlsx
+++ b/Projects_Section_Wise.xlsx
@@ -235,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -350,6 +350,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -5837,9 +5840,9 @@
           <t>Confirm hospital structure</t>
         </is>
       </c>
-      <c r="M58" s="40" t="inlineStr">
-        <is>
-          <t>In progress - session building now - frontend folder is empty; no requirements.txt / package.json; no entry point | 23 files NOT in git</t>
+      <c r="M58" s="25" t="inlineStr">
+        <is>
+          <t>Complete (code + README + run script + docs)</t>
         </is>
       </c>
     </row>
@@ -6038,9 +6041,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M61" s="40" t="inlineStr">
-        <is>
-          <t>In progress - session building now - no entry point | 19 files NOT in git</t>
+      <c r="M61" s="25" t="inlineStr">
+        <is>
+          <t>Complete (code + README + run script + docs)</t>
         </is>
       </c>
     </row>
@@ -6105,9 +6108,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M62" s="40" t="inlineStr">
-        <is>
-          <t>In progress - session building now - frontend folder is empty; no entry point | 17 files NOT in git</t>
+      <c r="M62" s="25" t="inlineStr">
+        <is>
+          <t>Complete (code + README + run script + docs)</t>
         </is>
       </c>
     </row>
@@ -6239,9 +6242,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M64" s="40" t="inlineStr">
-        <is>
-          <t>In progress - session building now - frontend folder is empty; no entry point | 20 files NOT in git</t>
+      <c r="M64" s="25" t="inlineStr">
+        <is>
+          <t>Complete (code + README + run script + docs)</t>
         </is>
       </c>
     </row>
@@ -6306,9 +6309,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M65" s="40" t="inlineStr">
-        <is>
-          <t>In progress - session building now - no entry point | 35 files NOT in git</t>
+      <c r="M65" s="25" t="inlineStr">
+        <is>
+          <t>Complete (code + README + run script + docs)</t>
         </is>
       </c>
     </row>
@@ -8491,7 +8494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18.28515625" customWidth="1" style="23" min="1" max="1"/>
@@ -8556,7 +8559,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D2" s="43" t="n">
+      <c r="D2" s="44" t="n">
         <v>534</v>
       </c>
       <c r="E2" s="30" t="inlineStr">
@@ -8569,7 +8572,7 @@
           <t>code + README + run script + docs | 286 files NOT in git</t>
         </is>
       </c>
-      <c r="G2" s="43" t="inlineStr">
+      <c r="G2" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8591,7 +8594,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D3" s="43" t="n">
+      <c r="D3" s="44" t="n">
         <v>28</v>
       </c>
       <c r="E3" s="32" t="inlineStr">
@@ -8604,7 +8607,7 @@
           <t>missing run/setup script, docs | 1 files NOT in git</t>
         </is>
       </c>
-      <c r="G3" s="43" t="inlineStr">
+      <c r="G3" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8626,7 +8629,7 @@
           <t>Testing Pending</t>
         </is>
       </c>
-      <c r="D4" s="43" t="n">
+      <c r="D4" s="44" t="n">
         <v>20</v>
       </c>
       <c r="E4" s="32" t="inlineStr">
@@ -8639,7 +8642,7 @@
           <t>missing run/setup script, docs | 1 .zip committed</t>
         </is>
       </c>
-      <c r="G4" s="43" t="inlineStr">
+      <c r="G4" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8661,7 +8664,7 @@
           <t>Testing Pending</t>
         </is>
       </c>
-      <c r="D5" s="43" t="n">
+      <c r="D5" s="44" t="n">
         <v>22</v>
       </c>
       <c r="E5" s="42" t="inlineStr">
@@ -8674,7 +8677,7 @@
           <t>session building now - missing run/setup script, docs | 1 .zip committed</t>
         </is>
       </c>
-      <c r="G5" s="43" t="inlineStr">
+      <c r="G5" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8692,7 +8695,7 @@
         </is>
       </c>
       <c r="C6" s="19" t="n"/>
-      <c r="D6" s="43" t="n">
+      <c r="D6" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="33" t="inlineStr">
@@ -8705,7 +8708,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G6" s="43" t="inlineStr">
+      <c r="G6" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8723,7 +8726,7 @@
         </is>
       </c>
       <c r="C7" s="19" t="n"/>
-      <c r="D7" s="43" t="n">
+      <c r="D7" s="44" t="n">
         <v>62</v>
       </c>
       <c r="E7" s="30" t="inlineStr">
@@ -8736,7 +8739,7 @@
           <t>code + README + run script + docs</t>
         </is>
       </c>
-      <c r="G7" s="43" t="inlineStr">
+      <c r="G7" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8754,7 +8757,7 @@
         </is>
       </c>
       <c r="C8" s="19" t="n"/>
-      <c r="D8" s="43" t="n">
+      <c r="D8" s="44" t="n">
         <v>75</v>
       </c>
       <c r="E8" s="30" t="inlineStr">
@@ -8767,7 +8770,7 @@
           <t>code + README + run script + docs</t>
         </is>
       </c>
-      <c r="G8" s="43" t="inlineStr">
+      <c r="G8" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8785,7 +8788,7 @@
         </is>
       </c>
       <c r="C9" s="19" t="n"/>
-      <c r="D9" s="43" t="n">
+      <c r="D9" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="33" t="inlineStr">
@@ -8798,7 +8801,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G9" s="43" t="inlineStr">
+      <c r="G9" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8816,7 +8819,7 @@
         </is>
       </c>
       <c r="C10" s="19" t="n"/>
-      <c r="D10" s="43" t="n">
+      <c r="D10" s="44" t="n">
         <v>19</v>
       </c>
       <c r="E10" s="34" t="inlineStr">
@@ -8829,7 +8832,7 @@
           <t>no requirements.txt / package.json | 1 .zip committed</t>
         </is>
       </c>
-      <c r="G10" s="43" t="inlineStr">
+      <c r="G10" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8847,7 +8850,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n"/>
-      <c r="D11" s="43" t="n">
+      <c r="D11" s="44" t="n">
         <v>84</v>
       </c>
       <c r="E11" s="32" t="inlineStr">
@@ -8860,7 +8863,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8878,7 +8881,7 @@
         </is>
       </c>
       <c r="C12" s="19" t="n"/>
-      <c r="D12" s="43" t="n">
+      <c r="D12" s="44" t="n">
         <v>106</v>
       </c>
       <c r="E12" s="32" t="inlineStr">
@@ -8891,7 +8894,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G12" s="43" t="inlineStr">
+      <c r="G12" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8909,7 +8912,7 @@
         </is>
       </c>
       <c r="C13" s="19" t="n"/>
-      <c r="D13" s="43" t="n">
+      <c r="D13" s="44" t="n">
         <v>3277</v>
       </c>
       <c r="E13" s="32" t="inlineStr">
@@ -8922,7 +8925,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G13" s="43" t="inlineStr">
+      <c r="G13" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8944,7 +8947,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D14" s="43" t="n">
+      <c r="D14" s="44" t="n">
         <v>238</v>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -8957,7 +8960,7 @@
           <t>code + README + run script + docs</t>
         </is>
       </c>
-      <c r="G14" s="43" t="inlineStr">
+      <c r="G14" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -8979,7 +8982,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D15" s="43" t="n">
+      <c r="D15" s="44" t="n">
         <v>17</v>
       </c>
       <c r="E15" s="42" t="inlineStr">
@@ -8992,7 +8995,7 @@
           <t>session building now - missing run/setup script, docs | 4 files NOT in git</t>
         </is>
       </c>
-      <c r="G15" s="43" t="inlineStr">
+      <c r="G15" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9010,7 +9013,7 @@
         </is>
       </c>
       <c r="C16" s="19" t="n"/>
-      <c r="D16" s="43" t="n">
+      <c r="D16" s="44" t="n">
         <v>87</v>
       </c>
       <c r="E16" s="32" t="inlineStr">
@@ -9023,7 +9026,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G16" s="43" t="inlineStr">
+      <c r="G16" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9041,7 +9044,7 @@
         </is>
       </c>
       <c r="C17" s="19" t="n"/>
-      <c r="D17" s="43" t="n">
+      <c r="D17" s="44" t="n">
         <v>31</v>
       </c>
       <c r="E17" s="34" t="inlineStr">
@@ -9054,7 +9057,7 @@
           <t>frontend folder is empty</t>
         </is>
       </c>
-      <c r="G17" s="43" t="inlineStr">
+      <c r="G17" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9072,7 +9075,7 @@
         </is>
       </c>
       <c r="C18" s="19" t="n"/>
-      <c r="D18" s="43" t="n">
+      <c r="D18" s="44" t="n">
         <v>145</v>
       </c>
       <c r="E18" s="32" t="inlineStr">
@@ -9085,7 +9088,7 @@
           <t>missing run/setup script, docs | 4 files NOT in git</t>
         </is>
       </c>
-      <c r="G18" s="43" t="inlineStr">
+      <c r="G18" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9108,7 +9111,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D20" s="43" t="n">
+      <c r="D20" s="44" t="n">
         <v>71</v>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -9121,7 +9124,7 @@
           <t>code + README + run script + docs | 4 files NOT in git</t>
         </is>
       </c>
-      <c r="G20" s="43" t="inlineStr">
+      <c r="G20" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9143,7 +9146,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D21" s="43" t="n">
+      <c r="D21" s="44" t="n">
         <v>399</v>
       </c>
       <c r="E21" s="30" t="inlineStr">
@@ -9156,7 +9159,7 @@
           <t>code + README + run script + docs | 7 files NOT in git</t>
         </is>
       </c>
-      <c r="G21" s="43" t="inlineStr">
+      <c r="G21" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9178,7 +9181,7 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="D22" s="43" t="n">
+      <c r="D22" s="44" t="n">
         <v>44</v>
       </c>
       <c r="E22" s="32" t="inlineStr">
@@ -9191,7 +9194,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G22" s="43" t="inlineStr">
+      <c r="G22" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9213,7 +9216,7 @@
           <t>Started</t>
         </is>
       </c>
-      <c r="D23" s="43" t="n">
+      <c r="D23" s="44" t="n">
         <v>352</v>
       </c>
       <c r="E23" s="30" t="inlineStr">
@@ -9226,7 +9229,7 @@
           <t>code + README + run script + docs | 11 files NOT in git</t>
         </is>
       </c>
-      <c r="G23" s="43" t="inlineStr">
+      <c r="G23" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9244,7 +9247,7 @@
         </is>
       </c>
       <c r="C24" s="19" t="n"/>
-      <c r="D24" s="43" t="n">
+      <c r="D24" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="33" t="inlineStr">
@@ -9257,7 +9260,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G24" s="43" t="inlineStr">
+      <c r="G24" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9275,7 +9278,7 @@
         </is>
       </c>
       <c r="C25" s="19" t="n"/>
-      <c r="D25" s="43" t="n">
+      <c r="D25" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="33" t="inlineStr">
@@ -9288,7 +9291,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G25" s="43" t="inlineStr">
+      <c r="G25" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9306,20 +9309,20 @@
         </is>
       </c>
       <c r="C26" s="19" t="n"/>
-      <c r="D26" s="43" t="n">
-        <v>23</v>
-      </c>
-      <c r="E26" s="42" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="D26" s="44" t="n">
+        <v>63</v>
+      </c>
+      <c r="E26" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="F26" s="31" t="inlineStr">
         <is>
-          <t>session building now - frontend folder is empty; no requirements.txt / package.json; no entry point | 23 files NOT in git</t>
-        </is>
-      </c>
-      <c r="G26" s="43" t="inlineStr">
+          <t>code + README + run script + docs | 1 files NOT in git</t>
+        </is>
+      </c>
+      <c r="G26" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9337,7 +9340,7 @@
         </is>
       </c>
       <c r="C27" s="19" t="n"/>
-      <c r="D27" s="43" t="n">
+      <c r="D27" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="33" t="inlineStr">
@@ -9350,7 +9353,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G27" s="43" t="inlineStr">
+      <c r="G27" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9368,7 +9371,7 @@
         </is>
       </c>
       <c r="C28" s="19" t="n"/>
-      <c r="D28" s="43" t="n">
+      <c r="D28" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -9381,7 +9384,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G28" s="43" t="inlineStr">
+      <c r="G28" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9399,20 +9402,20 @@
         </is>
       </c>
       <c r="C29" s="19" t="n"/>
-      <c r="D29" s="43" t="n">
-        <v>19</v>
-      </c>
-      <c r="E29" s="42" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="D29" s="44" t="n">
+        <v>210</v>
+      </c>
+      <c r="E29" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="F29" s="31" t="inlineStr">
         <is>
-          <t>session building now - no entry point | 19 files NOT in git</t>
-        </is>
-      </c>
-      <c r="G29" s="43" t="inlineStr">
+          <t>code + README + run script + docs | 15 files NOT in git</t>
+        </is>
+      </c>
+      <c r="G29" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9430,20 +9433,20 @@
         </is>
       </c>
       <c r="C30" s="19" t="n"/>
-      <c r="D30" s="43" t="n">
-        <v>17</v>
-      </c>
-      <c r="E30" s="42" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="D30" s="44" t="n">
+        <v>76</v>
+      </c>
+      <c r="E30" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="F30" s="31" t="inlineStr">
         <is>
-          <t>session building now - frontend folder is empty; no entry point | 17 files NOT in git</t>
-        </is>
-      </c>
-      <c r="G30" s="43" t="inlineStr">
+          <t>code + README + run script + docs | 5 files NOT in git</t>
+        </is>
+      </c>
+      <c r="G30" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9461,7 +9464,7 @@
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
-      <c r="D31" s="43" t="n">
+      <c r="D31" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="33" t="inlineStr">
@@ -9474,7 +9477,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G31" s="43" t="inlineStr">
+      <c r="G31" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9492,20 +9495,20 @@
         </is>
       </c>
       <c r="C32" s="19" t="n"/>
-      <c r="D32" s="43" t="n">
-        <v>20</v>
-      </c>
-      <c r="E32" s="42" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="D32" s="44" t="n">
+        <v>66</v>
+      </c>
+      <c r="E32" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="F32" s="31" t="inlineStr">
         <is>
-          <t>session building now - frontend folder is empty; no entry point | 20 files NOT in git</t>
-        </is>
-      </c>
-      <c r="G32" s="43" t="inlineStr">
+          <t>code + README + run script + docs | 2 files NOT in git</t>
+        </is>
+      </c>
+      <c r="G32" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9523,20 +9526,20 @@
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
-      <c r="D33" s="43" t="n">
-        <v>35</v>
-      </c>
-      <c r="E33" s="42" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
+      <c r="D33" s="44" t="n">
+        <v>82</v>
+      </c>
+      <c r="E33" s="30" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="F33" s="31" t="inlineStr">
         <is>
-          <t>session building now - no entry point | 35 files NOT in git</t>
-        </is>
-      </c>
-      <c r="G33" s="43" t="inlineStr">
+          <t>code + README + run script + docs | 2 files NOT in git</t>
+        </is>
+      </c>
+      <c r="G33" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9554,7 +9557,7 @@
         </is>
       </c>
       <c r="C34" s="19" t="n"/>
-      <c r="D34" s="43" t="n">
+      <c r="D34" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="33" t="inlineStr">
@@ -9567,7 +9570,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G34" s="43" t="inlineStr">
+      <c r="G34" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9585,7 +9588,7 @@
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
-      <c r="D35" s="43" t="n">
+      <c r="D35" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="33" t="inlineStr">
@@ -9598,7 +9601,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G35" s="43" t="inlineStr">
+      <c r="G35" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9616,7 +9619,7 @@
         </is>
       </c>
       <c r="C36" s="19" t="n"/>
-      <c r="D36" s="43" t="n">
+      <c r="D36" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E36" s="33" t="inlineStr">
@@ -9629,7 +9632,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G36" s="43" t="inlineStr">
+      <c r="G36" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9648,7 +9651,7 @@
         </is>
       </c>
       <c r="C38" s="19" t="n"/>
-      <c r="D38" s="43" t="n">
+      <c r="D38" s="44" t="n">
         <v>27</v>
       </c>
       <c r="E38" s="32" t="inlineStr">
@@ -9661,7 +9664,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G38" s="43" t="inlineStr">
+      <c r="G38" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9679,7 +9682,7 @@
         </is>
       </c>
       <c r="C39" s="19" t="n"/>
-      <c r="D39" s="43" t="n">
+      <c r="D39" s="44" t="n">
         <v>14</v>
       </c>
       <c r="E39" s="32" t="inlineStr">
@@ -9692,7 +9695,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G39" s="43" t="inlineStr">
+      <c r="G39" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9710,7 +9713,7 @@
         </is>
       </c>
       <c r="C40" s="19" t="n"/>
-      <c r="D40" s="43" t="n">
+      <c r="D40" s="44" t="n">
         <v>27</v>
       </c>
       <c r="E40" s="32" t="inlineStr">
@@ -9723,7 +9726,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G40" s="43" t="inlineStr">
+      <c r="G40" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9741,7 +9744,7 @@
         </is>
       </c>
       <c r="C41" s="19" t="n"/>
-      <c r="D41" s="43" t="n">
+      <c r="D41" s="44" t="n">
         <v>28</v>
       </c>
       <c r="E41" s="30" t="inlineStr">
@@ -9754,7 +9757,7 @@
           <t>code + README + run script + docs</t>
         </is>
       </c>
-      <c r="G41" s="43" t="inlineStr">
+      <c r="G41" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9772,7 +9775,7 @@
         </is>
       </c>
       <c r="C42" s="19" t="n"/>
-      <c r="D42" s="43" t="n">
+      <c r="D42" s="44" t="n">
         <v>34</v>
       </c>
       <c r="E42" s="32" t="inlineStr">
@@ -9785,7 +9788,7 @@
           <t>missing docs</t>
         </is>
       </c>
-      <c r="G42" s="43" t="inlineStr">
+      <c r="G42" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9803,7 +9806,7 @@
         </is>
       </c>
       <c r="C43" s="19" t="n"/>
-      <c r="D43" s="43" t="n">
+      <c r="D43" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="33" t="inlineStr">
@@ -9816,7 +9819,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G43" s="43" t="inlineStr">
+      <c r="G43" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9834,7 +9837,7 @@
         </is>
       </c>
       <c r="C44" s="19" t="n"/>
-      <c r="D44" s="43" t="n">
+      <c r="D44" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="33" t="inlineStr">
@@ -9847,7 +9850,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G44" s="43" t="inlineStr">
+      <c r="G44" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9865,7 +9868,7 @@
         </is>
       </c>
       <c r="C45" s="19" t="n"/>
-      <c r="D45" s="43" t="n">
+      <c r="D45" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="33" t="inlineStr">
@@ -9878,7 +9881,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G45" s="43" t="inlineStr">
+      <c r="G45" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9896,7 +9899,7 @@
         </is>
       </c>
       <c r="C46" s="19" t="n"/>
-      <c r="D46" s="43" t="n">
+      <c r="D46" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="33" t="inlineStr">
@@ -9909,7 +9912,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G46" s="43" t="inlineStr">
+      <c r="G46" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9927,7 +9930,7 @@
         </is>
       </c>
       <c r="C47" s="19" t="n"/>
-      <c r="D47" s="43" t="n">
+      <c r="D47" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="33" t="inlineStr">
@@ -9940,7 +9943,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G47" s="43" t="inlineStr">
+      <c r="G47" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9958,7 +9961,7 @@
         </is>
       </c>
       <c r="C48" s="19" t="n"/>
-      <c r="D48" s="43" t="n">
+      <c r="D48" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="33" t="inlineStr">
@@ -9971,7 +9974,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G48" s="43" t="inlineStr">
+      <c r="G48" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -9989,7 +9992,7 @@
         </is>
       </c>
       <c r="C49" s="19" t="n"/>
-      <c r="D49" s="43" t="n">
+      <c r="D49" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E49" s="33" t="inlineStr">
@@ -10002,7 +10005,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G49" s="43" t="inlineStr">
+      <c r="G49" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10020,7 +10023,7 @@
         </is>
       </c>
       <c r="C50" s="19" t="n"/>
-      <c r="D50" s="43" t="n">
+      <c r="D50" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E50" s="33" t="inlineStr">
@@ -10033,7 +10036,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G50" s="43" t="inlineStr">
+      <c r="G50" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10051,7 +10054,7 @@
         </is>
       </c>
       <c r="C51" s="19" t="n"/>
-      <c r="D51" s="43" t="n">
+      <c r="D51" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E51" s="33" t="inlineStr">
@@ -10064,7 +10067,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G51" s="43" t="inlineStr">
+      <c r="G51" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10082,7 +10085,7 @@
         </is>
       </c>
       <c r="C52" s="19" t="n"/>
-      <c r="D52" s="43" t="n">
+      <c r="D52" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E52" s="33" t="inlineStr">
@@ -10095,7 +10098,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G52" s="43" t="inlineStr">
+      <c r="G52" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10113,7 +10116,7 @@
         </is>
       </c>
       <c r="C53" s="19" t="n"/>
-      <c r="D53" s="43" t="n">
+      <c r="D53" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E53" s="33" t="inlineStr">
@@ -10126,7 +10129,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G53" s="43" t="inlineStr">
+      <c r="G53" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10144,7 +10147,7 @@
         </is>
       </c>
       <c r="C54" s="19" t="n"/>
-      <c r="D54" s="43" t="n">
+      <c r="D54" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E54" s="33" t="inlineStr">
@@ -10157,7 +10160,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G54" s="43" t="inlineStr">
+      <c r="G54" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10180,7 +10183,7 @@
         </is>
       </c>
       <c r="C56" s="19" t="n"/>
-      <c r="D56" s="43" t="n">
+      <c r="D56" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E56" s="33" t="inlineStr">
@@ -10193,7 +10196,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G56" s="43" t="inlineStr">
+      <c r="G56" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10211,7 +10214,7 @@
         </is>
       </c>
       <c r="C57" s="19" t="n"/>
-      <c r="D57" s="43" t="n">
+      <c r="D57" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E57" s="33" t="inlineStr">
@@ -10224,7 +10227,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G57" s="43" t="inlineStr">
+      <c r="G57" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10242,7 +10245,7 @@
         </is>
       </c>
       <c r="C58" s="19" t="n"/>
-      <c r="D58" s="43" t="n">
+      <c r="D58" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E58" s="33" t="inlineStr">
@@ -10255,7 +10258,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G58" s="43" t="inlineStr">
+      <c r="G58" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10273,7 +10276,7 @@
         </is>
       </c>
       <c r="C59" s="19" t="n"/>
-      <c r="D59" s="43" t="n">
+      <c r="D59" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E59" s="33" t="inlineStr">
@@ -10286,7 +10289,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G59" s="43" t="inlineStr">
+      <c r="G59" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10304,7 +10307,7 @@
         </is>
       </c>
       <c r="C60" s="19" t="n"/>
-      <c r="D60" s="43" t="n">
+      <c r="D60" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E60" s="33" t="inlineStr">
@@ -10317,7 +10320,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G60" s="43" t="inlineStr">
+      <c r="G60" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10335,7 +10338,7 @@
         </is>
       </c>
       <c r="C61" s="19" t="n"/>
-      <c r="D61" s="43" t="n">
+      <c r="D61" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E61" s="33" t="inlineStr">
@@ -10348,7 +10351,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G61" s="43" t="inlineStr">
+      <c r="G61" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10366,7 +10369,7 @@
         </is>
       </c>
       <c r="C62" s="19" t="n"/>
-      <c r="D62" s="43" t="n">
+      <c r="D62" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E62" s="33" t="inlineStr">
@@ -10379,7 +10382,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G62" s="43" t="inlineStr">
+      <c r="G62" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10397,7 +10400,7 @@
         </is>
       </c>
       <c r="C63" s="19" t="n"/>
-      <c r="D63" s="43" t="n">
+      <c r="D63" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E63" s="33" t="inlineStr">
@@ -10410,7 +10413,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G63" s="43" t="inlineStr">
+      <c r="G63" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10428,7 +10431,7 @@
         </is>
       </c>
       <c r="C64" s="19" t="n"/>
-      <c r="D64" s="43" t="n">
+      <c r="D64" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E64" s="33" t="inlineStr">
@@ -10441,7 +10444,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G64" s="43" t="inlineStr">
+      <c r="G64" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10459,7 +10462,7 @@
         </is>
       </c>
       <c r="C65" s="19" t="n"/>
-      <c r="D65" s="43" t="n">
+      <c r="D65" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E65" s="33" t="inlineStr">
@@ -10472,7 +10475,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G65" s="43" t="inlineStr">
+      <c r="G65" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10490,7 +10493,7 @@
         </is>
       </c>
       <c r="C66" s="19" t="n"/>
-      <c r="D66" s="43" t="n">
+      <c r="D66" s="44" t="n">
         <v>51</v>
       </c>
       <c r="E66" s="32" t="inlineStr">
@@ -10503,7 +10506,7 @@
           <t>missing run/setup script, docs</t>
         </is>
       </c>
-      <c r="G66" s="43" t="inlineStr">
+      <c r="G66" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10521,7 +10524,7 @@
         </is>
       </c>
       <c r="C67" s="19" t="n"/>
-      <c r="D67" s="43" t="n">
+      <c r="D67" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E67" s="33" t="inlineStr">
@@ -10534,7 +10537,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G67" s="43" t="inlineStr">
+      <c r="G67" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10552,7 +10555,7 @@
         </is>
       </c>
       <c r="C68" s="19" t="n"/>
-      <c r="D68" s="43" t="n">
+      <c r="D68" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E68" s="33" t="inlineStr">
@@ -10565,7 +10568,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G68" s="43" t="inlineStr">
+      <c r="G68" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10583,7 +10586,7 @@
         </is>
       </c>
       <c r="C69" s="19" t="n"/>
-      <c r="D69" s="43" t="n">
+      <c r="D69" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E69" s="33" t="inlineStr">
@@ -10596,7 +10599,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G69" s="43" t="inlineStr">
+      <c r="G69" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10614,7 +10617,7 @@
         </is>
       </c>
       <c r="C70" s="19" t="n"/>
-      <c r="D70" s="43" t="n">
+      <c r="D70" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E70" s="33" t="inlineStr">
@@ -10627,7 +10630,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G70" s="43" t="inlineStr">
+      <c r="G70" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10645,7 +10648,7 @@
         </is>
       </c>
       <c r="C71" s="19" t="n"/>
-      <c r="D71" s="43" t="n">
+      <c r="D71" s="44" t="n">
         <v>0</v>
       </c>
       <c r="E71" s="33" t="inlineStr">
@@ -10658,7 +10661,7 @@
           <t>only prompt + abstract</t>
         </is>
       </c>
-      <c r="G71" s="43" t="inlineStr">
+      <c r="G71" s="44" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -10984,6 +10987,7 @@
         <v>38</v>
       </c>
     </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="35" t="inlineStr">
         <is>
@@ -11150,6 +11154,175 @@
         <v>2</v>
       </c>
       <c r="G95" s="39" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="35" t="inlineStr">
+        <is>
+          <t>AUDIT SUMMARY (2026-09-28) - files present only; none of these have been run/tested</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="36" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B98" s="36" t="inlineStr">
+        <is>
+          <t>Batches</t>
+        </is>
+      </c>
+      <c r="C98" s="36" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="D98" s="36" t="inlineStr">
+        <is>
+          <t>IN PROGRESS</t>
+        </is>
+      </c>
+      <c r="E98" s="36" t="inlineStr">
+        <is>
+          <t>CODE ONLY</t>
+        </is>
+      </c>
+      <c r="F98" s="36" t="inlineStr">
+        <is>
+          <t>HAS GAPS</t>
+        </is>
+      </c>
+      <c r="G98" s="36" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="37" t="inlineStr">
+        <is>
+          <t>CSE-A</t>
+        </is>
+      </c>
+      <c r="B99" s="38" t="n">
+        <v>17</v>
+      </c>
+      <c r="C99" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="F99" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="38" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="37" t="inlineStr">
+        <is>
+          <t>CSE-C</t>
+        </is>
+      </c>
+      <c r="B100" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="C100" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D100" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="38" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="37" t="inlineStr">
+        <is>
+          <t>CSDS-A</t>
+        </is>
+      </c>
+      <c r="B101" s="38" t="n">
+        <v>17</v>
+      </c>
+      <c r="C101" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E101" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="F101" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" s="38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="37" t="inlineStr">
+        <is>
+          <t>CSDS-B</t>
+        </is>
+      </c>
+      <c r="B102" s="38" t="n">
+        <v>17</v>
+      </c>
+      <c r="C102" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="D102" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="38" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="39" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B103" s="39" t="n">
+        <v>67</v>
+      </c>
+      <c r="C103" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="D103" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="F103" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G103" s="39" t="n">
         <v>37</v>
       </c>
     </row>

</xml_diff>